<commit_message>
modified:   data.json 	modified:   ds.xlsx 	modified:   maybe first application i have made/data.json
</commit_message>
<xml_diff>
--- a/ds.xlsx
+++ b/ds.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DREAM ON\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04C648AB-548A-4B01-BC0E-C93504A7753D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B42A63FB-88F0-42AC-A10A-7CABEBF5878A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3180" yWindow="2810" windowWidth="14400" windowHeight="7270" xr2:uid="{BF172A33-4C81-4837-9283-885EE0BEB8A2}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BF172A33-4C81-4837-9283-885EE0BEB8A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>giahan.html</t>
   </si>
@@ -103,6 +103,12 @@
   </si>
   <si>
     <t>nhatlinh.html</t>
+  </si>
+  <si>
+    <t>0609</t>
+  </si>
+  <si>
+    <t>thiduong.html</t>
   </si>
 </sst>
 </file>
@@ -455,7 +461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7A91632-46E3-495F-8B1B-771380D56AAF}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="1"/>
@@ -574,6 +580,14 @@
         <v>25</v>
       </c>
     </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>